<commit_message>
feat: refine vendor onboarding and Linux release
</commit_message>
<xml_diff>
--- a/docs/农机配件平台_厂商产品资料采集模板.xlsx
+++ b/docs/农机配件平台_厂商产品资料采集模板.xlsx
@@ -218,7 +218,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AF3"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -253,8 +253,6 @@
     <col min="30" max="30" width="16" customWidth="1"/>
     <col min="31" max="31" width="16" customWidth="1"/>
     <col min="32" max="32" width="16" customWidth="1"/>
-    <col min="33" max="33" width="16" customWidth="1"/>
-    <col min="34" max="34" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -325,14 +323,14 @@
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">服务优势</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">主营产品</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">服务/适配机型</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">企业简介</t>
@@ -340,90 +338,80 @@
       </c>
       <c r="Q1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">服务优势</t>
+          <t xml:space="preserve">年产能/供货能力</t>
         </is>
       </c>
       <c r="R1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">年产能/供货能力</t>
+          <t xml:space="preserve">主要设备</t>
         </is>
       </c>
       <c r="S1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">主要设备</t>
+          <t xml:space="preserve">资质认证</t>
         </is>
       </c>
       <c r="T1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">资质认证</t>
+          <t xml:space="preserve">是否提供加工</t>
         </is>
       </c>
       <c r="U1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">售后服务</t>
+          <t xml:space="preserve">加工服务</t>
         </is>
       </c>
       <c r="V1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">是否提供加工</t>
+          <t xml:space="preserve">加工材料</t>
         </is>
       </c>
       <c r="W1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">加工服务</t>
+          <t xml:space="preserve">加工设备</t>
         </is>
       </c>
       <c r="X1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">加工材料</t>
+          <t xml:space="preserve">加工能力/精度</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">加工设备</t>
+          <t xml:space="preserve">服务区域</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">加工能力/精度</t>
+          <t xml:space="preserve">加工说明</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">服务区域</t>
+          <t xml:space="preserve">Logo URL</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">加工说明</t>
+          <t xml:space="preserve">封面图 URL</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Logo URL</t>
+          <t xml:space="preserve">发布状态</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">封面图 URL</t>
+          <t xml:space="preserve">推荐厂商</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">发布状态</t>
+          <t xml:space="preserve">平台认证</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">推荐厂商</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">平台认证</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">排序</t>
         </is>
@@ -497,14 +485,14 @@
       </c>
       <c r="N2" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">质量稳定、交付及时</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">齿轮、链条、液压件</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">拖拉机、收割机</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">企业简介示例</t>
@@ -512,90 +500,80 @@
       </c>
       <c r="Q2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">质量稳定、交付及时</t>
+          <t xml:space="preserve">年产20万套</t>
         </is>
       </c>
       <c r="R2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">年产20万套</t>
+          <t xml:space="preserve">数控车床、热处理设备</t>
         </is>
       </c>
       <c r="S2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">数控车床、热处理设备</t>
+          <t xml:space="preserve">ISO9001</t>
         </is>
       </c>
       <c r="T2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ISO9001</t>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
       <c r="U2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">质保12个月</t>
+          <t xml:space="preserve">来图加工、来样加工</t>
         </is>
       </c>
       <c r="V2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">是</t>
+          <t xml:space="preserve">45钢、铸铁</t>
         </is>
       </c>
       <c r="W2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">来图加工、来样加工</t>
+          <t xml:space="preserve">数控车床、磨床</t>
         </is>
       </c>
       <c r="X2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">45钢、铸铁</t>
+          <t xml:space="preserve">轴类±0.02mm</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">数控车床、磨床</t>
+          <t xml:space="preserve">华北地区</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">轴类±0.02mm</t>
+          <t xml:space="preserve">支持小批量定制</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">华北地区</t>
+          <t xml:space="preserve">https://vendor.example.cn/logo.png</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">支持小批量定制</t>
+          <t xml:space="preserve">https://vendor.example.cn/cover.jpg</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">https://vendor.example.cn/logo.png</t>
+          <t xml:space="preserve">隐藏</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">https://vendor.example.cn/cover.jpg</t>
+          <t xml:space="preserve">否</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">隐藏</t>
+          <t xml:space="preserve">否</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">否</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">否</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">100</t>
         </is>
@@ -762,27 +740,17 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="AG3" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH2000"/>
+  <autoFilter ref="A1:AF2000"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="填写值无效" error="请从下拉列表中选择" sqref="V2:V2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="填写值无效" error="请从下拉列表中选择" sqref="T2:T2000">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="填写值无效" error="请从下拉列表中选择" sqref="AE2:AE2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="填写值无效" error="请从下拉列表中选择" sqref="AC2:AC2000">
       <formula1>"草稿,已发布,隐藏"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="填写值无效" error="请从下拉列表中选择" sqref="AF2:AG2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="填写值无效" error="请从下拉列表中选择" sqref="AD2:AE2000">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>